<commit_message>
feat: update config and department mapping integration
</commit_message>
<xml_diff>
--- a/data/11506/系所經費代碼與中文名稱對照表.xlsx
+++ b/data/11506/系所經費代碼與中文名稱對照表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\IR大數據分析組\IR-躍升相關\經費收支明細\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB5E34F6-0ECE-4BE5-817C-CFB69C70361F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC8DD0A-16FF-4247-8365-BF14617CED58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A410AB86-5814-4FCF-ADFA-7EA48B0B568D}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="116">
   <si>
     <r>
       <rPr>
@@ -237,10 +237,6 @@
       </rPr>
       <t>半導體工程系</t>
     </r>
-  </si>
-  <si>
-    <t>UB03</t>
-    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -996,6 +992,116 @@
   </si>
   <si>
     <t>UF02</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>UB00</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>UD01</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>新增</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>GB00</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>漁業科技與管理系</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>環安衛</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>UT00</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>UV00</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>YE00</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="標楷體"/>
+        <family val="4"/>
+        <charset val="136"/>
+      </rPr>
+      <t>海洋休閒管理系</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>綜業</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>)</t>
+    </r>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1003,7 +1109,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1038,6 +1144,26 @@
       <name val="Times New Roman"/>
       <family val="4"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Times New Roman"/>
+      <family val="4"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="4"/>
+      <charset val="136"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1241,27 +1367,9 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1291,6 +1399,30 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1607,545 +1739,612 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D452D504-C59B-4FEE-9796-EA0E20A0674F}">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="6"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="16"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="6" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="17" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="C10" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="12" t="s">
+      <c r="B11" s="5" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
+      <c r="C11" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="12" t="s">
+      <c r="B14" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="12" t="s">
+      <c r="B18" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+      <c r="B24" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
+      <c r="B25" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="D27" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B15" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+      <c r="B28" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="D31" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="B34" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C41" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="D41" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C18" s="12" t="s">
+      <c r="B42" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B43" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="C43" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="D43" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="4" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+      <c r="B45" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B26" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B27" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B30" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C30" s="12" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B31" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="C31" s="12" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C32" s="12" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B34" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B35" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B36" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="C36" s="12" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B37" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="C37" s="12" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B38" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="C38" s="12" t="s">
+      <c r="B46" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="4" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="B39" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="C39" s="12" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B40" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="C40" s="12" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B41" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="C41" s="12" t="s">
+      <c r="B47" s="5" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="B42" s="11" t="s">
+      <c r="C47" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C42" s="12" t="s">
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B48" s="5" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="B43" s="11" t="s">
+      <c r="C48" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="C43" s="12" t="s">
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="4" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="10" t="s">
+      <c r="B49" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B44" s="11" t="s">
+      <c r="C49" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C44" s="12" t="s">
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B50" s="5" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="B45" s="11" t="s">
+      <c r="C50" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="C45" s="12" t="s">
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B51" s="5" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="B46" s="11" t="s">
+      <c r="C51" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="C46" s="12" t="s">
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B52" s="5" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="10" t="s">
+      <c r="C52" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B47" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="C47" s="12" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B48" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="C48" s="12" t="s">
+      <c r="B54" s="9" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="B49" s="15" t="s">
+      <c r="C54" s="10" t="s">
         <v>106</v>
-      </c>
-      <c r="C49" s="16" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>